<commit_message>
chore: refresh generated dashboards + fleet control sheet
Regenerated artifacts (derive from fleet-status.md):
- dashboard.html, morning-brief.html
- OBB Fleet Control Sheet xlsx (minor re-save)

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ND-DEL-OBB-035-CFG-001-01 OBB Fleet Control Sheet 20260211.xlsx
+++ b/ND-DEL-OBB-035-CFG-001-01 OBB Fleet Control Sheet 20260211.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AbbasRizvi\Documents\dosto-troubleshooting\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AEACCCED-7295-41A9-839D-8A34DA6DD779}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABB214A4-6770-4C13-B58F-565A691FC698}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="4" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="830" uniqueCount="318">
   <si>
     <t>Issued To:</t>
   </si>
@@ -1031,6 +1031,9 @@
   </si>
   <si>
     <t>Punchlist</t>
+  </si>
+  <si>
+    <t>10.179.41.1</t>
   </si>
 </sst>
 </file>
@@ -2456,51 +2459,78 @@
     <xf numFmtId="0" fontId="29" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="3" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="3" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="121" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="121" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="121" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="121" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="121" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="7" xfId="121" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="121" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="2" borderId="8" xfId="121" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="121" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="121" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="121" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="8" xfId="121" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -2513,37 +2543,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="121" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="121" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="121" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="121" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="7" xfId="121" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="0" xfId="121" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="2" borderId="8" xfId="121" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="121" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="121" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="121" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="14" fontId="4" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="3" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3334,9 +3337,9 @@
       <c r="E1" s="7"/>
       <c r="F1" s="7"/>
       <c r="G1" s="7"/>
-      <c r="H1" s="141"/>
-      <c r="I1" s="141"/>
-      <c r="J1" s="141"/>
+      <c r="H1" s="137"/>
+      <c r="I1" s="137"/>
+      <c r="J1" s="137"/>
       <c r="K1" s="7"/>
       <c r="L1" s="7"/>
       <c r="M1" s="8"/>
@@ -3533,21 +3536,21 @@
       <c r="M12" s="11"/>
     </row>
     <row r="13" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A13" s="142" t="s">
+      <c r="A13" s="138" t="s">
         <v>10</v>
       </c>
-      <c r="B13" s="143"/>
-      <c r="C13" s="143"/>
-      <c r="D13" s="143"/>
-      <c r="E13" s="143"/>
-      <c r="F13" s="143"/>
-      <c r="G13" s="143"/>
-      <c r="H13" s="143"/>
-      <c r="I13" s="143"/>
-      <c r="J13" s="143"/>
-      <c r="K13" s="143"/>
-      <c r="L13" s="143"/>
-      <c r="M13" s="144"/>
+      <c r="B13" s="139"/>
+      <c r="C13" s="139"/>
+      <c r="D13" s="139"/>
+      <c r="E13" s="139"/>
+      <c r="F13" s="139"/>
+      <c r="G13" s="139"/>
+      <c r="H13" s="139"/>
+      <c r="I13" s="139"/>
+      <c r="J13" s="139"/>
+      <c r="K13" s="139"/>
+      <c r="L13" s="139"/>
+      <c r="M13" s="140"/>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A14" s="9"/>
@@ -3627,48 +3630,48 @@
       <c r="M18" s="11"/>
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A19" s="139"/>
-      <c r="B19" s="140"/>
-      <c r="C19" s="140"/>
-      <c r="D19" s="140"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="140"/>
-      <c r="G19" s="140"/>
-      <c r="H19" s="140"/>
-      <c r="I19" s="140"/>
-      <c r="J19" s="140"/>
-      <c r="K19" s="140"/>
-      <c r="L19" s="140"/>
+      <c r="A19" s="135"/>
+      <c r="B19" s="136"/>
+      <c r="C19" s="136"/>
+      <c r="D19" s="136"/>
+      <c r="E19" s="136"/>
+      <c r="F19" s="136"/>
+      <c r="G19" s="136"/>
+      <c r="H19" s="136"/>
+      <c r="I19" s="136"/>
+      <c r="J19" s="136"/>
+      <c r="K19" s="136"/>
+      <c r="L19" s="136"/>
       <c r="M19" s="11"/>
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A20" s="139"/>
-      <c r="B20" s="140"/>
-      <c r="C20" s="140"/>
-      <c r="D20" s="140"/>
-      <c r="E20" s="140"/>
-      <c r="F20" s="140"/>
-      <c r="G20" s="140"/>
-      <c r="H20" s="140"/>
-      <c r="I20" s="140"/>
-      <c r="J20" s="140"/>
-      <c r="K20" s="140"/>
-      <c r="L20" s="140"/>
+      <c r="A20" s="135"/>
+      <c r="B20" s="136"/>
+      <c r="C20" s="136"/>
+      <c r="D20" s="136"/>
+      <c r="E20" s="136"/>
+      <c r="F20" s="136"/>
+      <c r="G20" s="136"/>
+      <c r="H20" s="136"/>
+      <c r="I20" s="136"/>
+      <c r="J20" s="136"/>
+      <c r="K20" s="136"/>
+      <c r="L20" s="136"/>
       <c r="M20" s="11"/>
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A21" s="139"/>
-      <c r="B21" s="140"/>
-      <c r="C21" s="140"/>
-      <c r="D21" s="140"/>
-      <c r="E21" s="140"/>
-      <c r="F21" s="140"/>
-      <c r="G21" s="140"/>
-      <c r="H21" s="140"/>
-      <c r="I21" s="140"/>
-      <c r="J21" s="140"/>
-      <c r="K21" s="140"/>
-      <c r="L21" s="140"/>
+      <c r="A21" s="135"/>
+      <c r="B21" s="136"/>
+      <c r="C21" s="136"/>
+      <c r="D21" s="136"/>
+      <c r="E21" s="136"/>
+      <c r="F21" s="136"/>
+      <c r="G21" s="136"/>
+      <c r="H21" s="136"/>
+      <c r="I21" s="136"/>
+      <c r="J21" s="136"/>
+      <c r="K21" s="136"/>
+      <c r="L21" s="136"/>
       <c r="M21" s="11"/>
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.2">
@@ -3734,21 +3737,21 @@
       <c r="M25" s="11"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A26" s="145" t="s">
+      <c r="A26" s="141" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="146"/>
-      <c r="C26" s="146"/>
-      <c r="D26" s="146"/>
-      <c r="E26" s="146"/>
-      <c r="F26" s="146"/>
-      <c r="G26" s="146"/>
-      <c r="H26" s="146"/>
-      <c r="I26" s="146"/>
-      <c r="J26" s="146"/>
-      <c r="K26" s="146"/>
-      <c r="L26" s="146"/>
-      <c r="M26" s="147"/>
+      <c r="B26" s="142"/>
+      <c r="C26" s="142"/>
+      <c r="D26" s="142"/>
+      <c r="E26" s="142"/>
+      <c r="F26" s="142"/>
+      <c r="G26" s="142"/>
+      <c r="H26" s="142"/>
+      <c r="I26" s="142"/>
+      <c r="J26" s="142"/>
+      <c r="K26" s="142"/>
+      <c r="L26" s="142"/>
+      <c r="M26" s="143"/>
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A27" s="133"/>
@@ -3763,7 +3766,7 @@
       <c r="J27" s="134"/>
       <c r="K27" s="134"/>
       <c r="L27" s="134"/>
-      <c r="M27" s="135"/>
+      <c r="M27" s="144"/>
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A28" s="133"/>
@@ -3793,7 +3796,7 @@
       <c r="J29" s="134"/>
       <c r="K29" s="134"/>
       <c r="L29" s="134"/>
-      <c r="M29" s="135"/>
+      <c r="M29" s="144"/>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A30" s="133"/>
@@ -3808,7 +3811,7 @@
       <c r="J30" s="134"/>
       <c r="K30" s="134"/>
       <c r="L30" s="134"/>
-      <c r="M30" s="135"/>
+      <c r="M30" s="144"/>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A31" s="133"/>
@@ -3823,7 +3826,7 @@
       <c r="J31" s="134"/>
       <c r="K31" s="134"/>
       <c r="L31" s="134"/>
-      <c r="M31" s="135"/>
+      <c r="M31" s="144"/>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A32" s="133"/>
@@ -3838,64 +3841,64 @@
       <c r="J32" s="134"/>
       <c r="K32" s="134"/>
       <c r="L32" s="134"/>
-      <c r="M32" s="135"/>
+      <c r="M32" s="144"/>
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A33" s="136"/>
-      <c r="B33" s="137"/>
-      <c r="C33" s="137"/>
-      <c r="D33" s="137"/>
-      <c r="E33" s="137"/>
-      <c r="F33" s="137"/>
-      <c r="G33" s="137"/>
-      <c r="H33" s="137"/>
-      <c r="I33" s="137"/>
-      <c r="J33" s="137"/>
+      <c r="A33" s="145"/>
+      <c r="B33" s="146"/>
+      <c r="C33" s="146"/>
+      <c r="D33" s="146"/>
+      <c r="E33" s="146"/>
+      <c r="F33" s="146"/>
+      <c r="G33" s="146"/>
+      <c r="H33" s="146"/>
+      <c r="I33" s="146"/>
+      <c r="J33" s="146"/>
       <c r="K33" s="10"/>
       <c r="L33" s="10"/>
       <c r="M33" s="11"/>
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A34" s="138"/>
-      <c r="B34" s="137"/>
-      <c r="C34" s="137"/>
-      <c r="D34" s="137"/>
-      <c r="E34" s="137"/>
-      <c r="F34" s="137"/>
-      <c r="G34" s="137"/>
-      <c r="H34" s="137"/>
-      <c r="I34" s="137"/>
-      <c r="J34" s="137"/>
+      <c r="A34" s="147"/>
+      <c r="B34" s="146"/>
+      <c r="C34" s="146"/>
+      <c r="D34" s="146"/>
+      <c r="E34" s="146"/>
+      <c r="F34" s="146"/>
+      <c r="G34" s="146"/>
+      <c r="H34" s="146"/>
+      <c r="I34" s="146"/>
+      <c r="J34" s="146"/>
       <c r="K34" s="10"/>
       <c r="L34" s="10"/>
       <c r="M34" s="11"/>
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A35" s="138"/>
-      <c r="B35" s="137"/>
-      <c r="C35" s="137"/>
-      <c r="D35" s="137"/>
-      <c r="E35" s="137"/>
-      <c r="F35" s="137"/>
-      <c r="G35" s="137"/>
-      <c r="H35" s="137"/>
-      <c r="I35" s="137"/>
-      <c r="J35" s="137"/>
+      <c r="A35" s="147"/>
+      <c r="B35" s="146"/>
+      <c r="C35" s="146"/>
+      <c r="D35" s="146"/>
+      <c r="E35" s="146"/>
+      <c r="F35" s="146"/>
+      <c r="G35" s="146"/>
+      <c r="H35" s="146"/>
+      <c r="I35" s="146"/>
+      <c r="J35" s="146"/>
       <c r="K35" s="10"/>
       <c r="L35" s="10"/>
       <c r="M35" s="11"/>
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.2">
-      <c r="A36" s="138"/>
-      <c r="B36" s="137"/>
-      <c r="C36" s="137"/>
-      <c r="D36" s="137"/>
-      <c r="E36" s="137"/>
-      <c r="F36" s="137"/>
-      <c r="G36" s="137"/>
-      <c r="H36" s="137"/>
-      <c r="I36" s="137"/>
-      <c r="J36" s="137"/>
+      <c r="A36" s="147"/>
+      <c r="B36" s="146"/>
+      <c r="C36" s="146"/>
+      <c r="D36" s="146"/>
+      <c r="E36" s="146"/>
+      <c r="F36" s="146"/>
+      <c r="G36" s="146"/>
+      <c r="H36" s="146"/>
+      <c r="I36" s="146"/>
+      <c r="J36" s="146"/>
       <c r="K36" s="10"/>
       <c r="L36" s="10"/>
       <c r="M36" s="11"/>
@@ -3932,17 +3935,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A29:M29"/>
+    <mergeCell ref="A30:M30"/>
+    <mergeCell ref="A31:M31"/>
+    <mergeCell ref="A32:M32"/>
+    <mergeCell ref="A33:J36"/>
     <mergeCell ref="A28:L28"/>
     <mergeCell ref="A19:L21"/>
     <mergeCell ref="H1:J1"/>
     <mergeCell ref="A13:M13"/>
     <mergeCell ref="A26:M26"/>
     <mergeCell ref="A27:M27"/>
-    <mergeCell ref="A29:M29"/>
-    <mergeCell ref="A30:M30"/>
-    <mergeCell ref="A31:M31"/>
-    <mergeCell ref="A32:M32"/>
-    <mergeCell ref="A33:J36"/>
   </mergeCells>
   <pageMargins left="0.70866141732283472" right="0.70866141732283472" top="0.74803149606299213" bottom="0.74803149606299213" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="84" orientation="landscape" r:id="rId1"/>
@@ -3987,11 +3990,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="120" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
       <c r="D1" s="23"/>
       <c r="E1" s="49"/>
       <c r="F1" s="50"/>
@@ -4004,70 +4007,70 @@
       <c r="M1" s="17"/>
     </row>
     <row r="2" spans="1:17" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="130" t="s">
+      <c r="B2" s="128" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="128" t="s">
+      <c r="C2" s="126" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="131" t="s">
+      <c r="D2" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="123" t="s">
+      <c r="E2" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="124" t="s">
+      <c r="F2" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="123" t="s">
+      <c r="G2" s="124" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="123" t="s">
+      <c r="H2" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="123" t="s">
+      <c r="I2" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="123" t="s">
+      <c r="J2" s="124" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="125" t="s">
+      <c r="K2" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="125" t="s">
+      <c r="L2" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="125" t="s">
+      <c r="M2" s="122" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="123" t="s">
+      <c r="N2" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="123" t="s">
+      <c r="O2" s="124" t="s">
         <v>29</v>
       </c>
       <c r="P2" s="19"/>
       <c r="Q2" s="19"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="129"/>
-      <c r="B3" s="131"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="149"/>
-      <c r="E3" s="124"/>
-      <c r="F3" s="148"/>
-      <c r="G3" s="124"/>
-      <c r="H3" s="124"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="125"/>
-      <c r="L3" s="125"/>
-      <c r="M3" s="125"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
+      <c r="A3" s="127"/>
+      <c r="B3" s="129"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="125"/>
+      <c r="F3" s="149"/>
+      <c r="G3" s="125"/>
+      <c r="H3" s="125"/>
+      <c r="I3" s="124"/>
+      <c r="J3" s="124"/>
+      <c r="K3" s="122"/>
+      <c r="L3" s="122"/>
+      <c r="M3" s="122"/>
+      <c r="N3" s="124"/>
+      <c r="O3" s="124"/>
       <c r="P3" s="22"/>
       <c r="Q3" s="19"/>
     </row>
@@ -6121,12 +6124,6 @@
     </sortState>
   </autoFilter>
   <mergeCells count="16">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="N2:N3"/>
@@ -6137,6 +6134,12 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -6171,11 +6174,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="120" t="s">
         <v>31</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
       <c r="D1" s="23"/>
       <c r="E1" s="49"/>
       <c r="F1" s="50"/>
@@ -6188,70 +6191,70 @@
       <c r="M1" s="17"/>
     </row>
     <row r="2" spans="1:17" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="130" t="s">
+      <c r="B2" s="128" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="128" t="s">
+      <c r="C2" s="126" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="131" t="s">
+      <c r="D2" s="129" t="s">
         <v>18</v>
       </c>
-      <c r="E2" s="123" t="s">
+      <c r="E2" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="F2" s="124" t="s">
+      <c r="F2" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="G2" s="123" t="s">
+      <c r="G2" s="124" t="s">
         <v>21</v>
       </c>
-      <c r="H2" s="123" t="s">
+      <c r="H2" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="I2" s="123" t="s">
+      <c r="I2" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="J2" s="123" t="s">
+      <c r="J2" s="124" t="s">
         <v>24</v>
       </c>
-      <c r="K2" s="125" t="s">
+      <c r="K2" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="L2" s="125" t="s">
+      <c r="L2" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="M2" s="125" t="s">
+      <c r="M2" s="122" t="s">
         <v>27</v>
       </c>
-      <c r="N2" s="123" t="s">
+      <c r="N2" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="O2" s="123" t="s">
+      <c r="O2" s="124" t="s">
         <v>29</v>
       </c>
       <c r="P2" s="19"/>
       <c r="Q2" s="19"/>
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
-      <c r="A3" s="129"/>
-      <c r="B3" s="131"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="149"/>
-      <c r="E3" s="124"/>
-      <c r="F3" s="148"/>
-      <c r="G3" s="124"/>
-      <c r="H3" s="124"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="125"/>
-      <c r="L3" s="125"/>
-      <c r="M3" s="125"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
+      <c r="A3" s="127"/>
+      <c r="B3" s="129"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="148"/>
+      <c r="E3" s="125"/>
+      <c r="F3" s="149"/>
+      <c r="G3" s="125"/>
+      <c r="H3" s="125"/>
+      <c r="I3" s="124"/>
+      <c r="J3" s="124"/>
+      <c r="K3" s="122"/>
+      <c r="L3" s="122"/>
+      <c r="M3" s="122"/>
+      <c r="N3" s="124"/>
+      <c r="O3" s="124"/>
       <c r="P3" s="22"/>
       <c r="Q3" s="19"/>
     </row>
@@ -8305,12 +8308,6 @@
     </sortState>
   </autoFilter>
   <mergeCells count="16">
-    <mergeCell ref="E2:E3"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-    <mergeCell ref="D2:D3"/>
     <mergeCell ref="L2:L3"/>
     <mergeCell ref="M2:M3"/>
     <mergeCell ref="N2:N3"/>
@@ -8321,6 +8318,12 @@
     <mergeCell ref="I2:I3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="K2:K3"/>
+    <mergeCell ref="E2:E3"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:A3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -8355,11 +8358,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="126" t="s">
+      <c r="A1" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="B1" s="127"/>
-      <c r="C1" s="127"/>
+      <c r="B1" s="121"/>
+      <c r="C1" s="121"/>
       <c r="D1" s="49"/>
       <c r="E1" s="50"/>
       <c r="F1" s="20"/>
@@ -8375,58 +8378,58 @@
       <c r="P1" s="61"/>
     </row>
     <row r="2" spans="1:20" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="128" t="s">
+      <c r="A2" s="126" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="130" t="s">
+      <c r="B2" s="128" t="s">
         <v>16</v>
       </c>
-      <c r="C2" s="128" t="s">
+      <c r="C2" s="126" t="s">
         <v>17</v>
       </c>
-      <c r="D2" s="123" t="s">
+      <c r="D2" s="124" t="s">
         <v>19</v>
       </c>
-      <c r="E2" s="124" t="s">
+      <c r="E2" s="125" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="123" t="s">
+      <c r="F2" s="124" t="s">
         <v>21</v>
       </c>
-      <c r="G2" s="123" t="s">
+      <c r="G2" s="124" t="s">
         <v>22</v>
       </c>
-      <c r="H2" s="123" t="s">
+      <c r="H2" s="124" t="s">
         <v>23</v>
       </c>
-      <c r="I2" s="123" t="s">
+      <c r="I2" s="124" t="s">
         <v>24</v>
       </c>
-      <c r="J2" s="125" t="s">
+      <c r="J2" s="122" t="s">
         <v>25</v>
       </c>
-      <c r="K2" s="120" t="s">
+      <c r="K2" s="123" t="s">
         <v>33</v>
       </c>
-      <c r="L2" s="120" t="s">
+      <c r="L2" s="123" t="s">
         <v>34</v>
       </c>
       <c r="M2" s="101" t="s">
         <v>35</v>
       </c>
-      <c r="N2" s="120" t="s">
+      <c r="N2" s="123" t="s">
         <v>36</v>
       </c>
-      <c r="O2" s="125" t="s">
+      <c r="O2" s="122" t="s">
         <v>26</v>
       </c>
-      <c r="P2" s="125" t="s">
+      <c r="P2" s="122" t="s">
         <v>27</v>
       </c>
-      <c r="Q2" s="123" t="s">
+      <c r="Q2" s="124" t="s">
         <v>28</v>
       </c>
-      <c r="R2" s="123" t="s">
+      <c r="R2" s="124" t="s">
         <v>29</v>
       </c>
       <c r="S2" s="19"/>
@@ -8435,24 +8438,24 @@
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A3" s="129"/>
-      <c r="B3" s="131"/>
-      <c r="C3" s="129"/>
-      <c r="D3" s="124"/>
-      <c r="E3" s="132"/>
-      <c r="F3" s="124"/>
-      <c r="G3" s="124"/>
-      <c r="H3" s="124"/>
-      <c r="I3" s="124"/>
-      <c r="J3" s="120"/>
-      <c r="K3" s="122"/>
-      <c r="L3" s="122"/>
+      <c r="A3" s="127"/>
+      <c r="B3" s="129"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="125"/>
+      <c r="E3" s="130"/>
+      <c r="F3" s="125"/>
+      <c r="G3" s="125"/>
+      <c r="H3" s="125"/>
+      <c r="I3" s="125"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="132"/>
+      <c r="L3" s="132"/>
       <c r="M3" s="100"/>
-      <c r="N3" s="121"/>
-      <c r="O3" s="120"/>
-      <c r="P3" s="120"/>
-      <c r="Q3" s="124"/>
-      <c r="R3" s="124"/>
+      <c r="N3" s="131"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="125"/>
+      <c r="R3" s="125"/>
       <c r="S3" s="22"/>
       <c r="T3" s="19"/>
     </row>
@@ -11429,7 +11432,7 @@
       </c>
       <c r="I81" s="30"/>
       <c r="J81" s="97" t="s">
-        <v>306</v>
+        <v>317</v>
       </c>
       <c r="K81" s="75" t="s">
         <v>44</v>
@@ -11988,6 +11991,13 @@
     </sortState>
   </autoFilter>
   <mergeCells count="18">
+    <mergeCell ref="N2:N3"/>
+    <mergeCell ref="K2:K3"/>
+    <mergeCell ref="L2:L3"/>
+    <mergeCell ref="R2:R3"/>
+    <mergeCell ref="Q2:Q3"/>
+    <mergeCell ref="P2:P3"/>
+    <mergeCell ref="O2:O3"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="I2:I3"/>
@@ -11999,13 +12009,6 @@
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="A2:A3"/>
     <mergeCell ref="E2:E3"/>
-    <mergeCell ref="N2:N3"/>
-    <mergeCell ref="K2:K3"/>
-    <mergeCell ref="L2:L3"/>
-    <mergeCell ref="R2:R3"/>
-    <mergeCell ref="Q2:Q3"/>
-    <mergeCell ref="P2:P3"/>
-    <mergeCell ref="O2:O3"/>
   </mergeCells>
   <phoneticPr fontId="31" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12015,15 +12018,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F95E44EFD72B924DB5304C1CB5281D76" ma:contentTypeVersion="" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1ba9161c84d20e2ccfd9d6939919cfea">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="ae9c23e9-1d64-4f26-b096-e89c4e22b406" xmlns:ns3="94c78f62-2d8e-4b44-a6a6-1d05c154aadf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4d289a11da5f0aaf1b4f088659dcbc38" ns2:_="" ns3:_="">
     <xsd:import namespace="ae9c23e9-1d64-4f26-b096-e89c4e22b406"/>
@@ -12252,6 +12246,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -12264,14 +12267,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD22EE22-6923-4830-A493-C3302739F86B}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C4F725D-6DD9-4DD5-A1FE-7E4E5610E547}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -12286,6 +12281,14 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD22EE22-6923-4830-A493-C3302739F86B}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>